<commit_message>
Combine CMouse. Separate Define.mqh
</commit_message>
<xml_diff>
--- a/Experts/Anhnt/Document/MQL5 Note/MouseCombine.xlsx
+++ b/Experts/Anhnt/Document/MQL5 Note/MouseCombine.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\AppData\Roaming\MetaQuotes\Terminal\D0E8209F77C8CF37AD8BF550E51FF075\MQL5\Experts\Anhnt\Document\MQL5 Note\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BBB07C2-33C0-4817-904A-A7752D80F7F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71433986-03F1-41CF-8C1C-115C946B8C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{025EE299-CAF2-4F37-A6EF-2D1360028262}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{025EE299-CAF2-4F37-A6EF-2D1360028262}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Compare 3 Class" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="232">
   <si>
     <r>
       <t xml:space="preserve">Về lý thuyết thì được, nhưng cần cẩn thận vì </t>
@@ -856,12 +857,222 @@
   <si>
     <t>down_thick_black</t>
   </si>
+  <si>
+    <t>Fields</t>
+  </si>
+  <si>
+    <t>CMouseCombine hiện tại</t>
+  </si>
+  <si>
+    <t>Nên dùng</t>
+  </si>
+  <si>
+    <t>m_x</t>
+  </si>
+  <si>
+    <t>m_coord_x</t>
+  </si>
+  <si>
+    <r>
+      <t>m_x</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="163"/>
+      </rPr>
+      <t> (CMouse) ✓</t>
+    </r>
+  </si>
+  <si>
+    <t>m_y</t>
+  </si>
+  <si>
+    <t>m_coord_y</t>
+  </si>
+  <si>
+    <r>
+      <t>m_y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="163"/>
+      </rPr>
+      <t> (CMouse) ✓</t>
+    </r>
+  </si>
+  <si>
+    <t>m_subwin</t>
+  </si>
+  <si>
+    <r>
+      <t>m_subwin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF616161"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+        <charset val="163"/>
+      </rPr>
+      <t> (CMouse) ✓</t>
+    </r>
+  </si>
+  <si>
+    <t>m_time</t>
+  </si>
+  <si>
+    <t>✓</t>
+  </si>
+  <si>
+    <t>m_level</t>
+  </si>
+  <si>
+    <t>m_call_counter</t>
+  </si>
+  <si>
+    <t>m_delta_wheel</t>
+  </si>
+  <si>
+    <t>m_state_flags</t>
+  </si>
+  <si>
+    <t>m_left_button_state</t>
+  </si>
+  <si>
+    <t>Cần thêm</t>
+  </si>
+  <si>
+    <t>m_pause_between_clicks</t>
+  </si>
+  <si>
+    <t>Methods — cần đổi tên</t>
+  </si>
+  <si>
+    <t>Vấn đề</t>
+  </si>
+  <si>
+    <t>Tên sai, đổi lại</t>
+  </si>
+  <si>
+    <t>IsPressedButtonRight()</t>
+  </si>
+  <si>
+    <t>IsRightBtn()</t>
+  </si>
+  <si>
+    <t>Tên sai</t>
+  </si>
+  <si>
+    <t>IsPressedButtonMiddle()</t>
+  </si>
+  <si>
+    <t>IsMiddleBtn()</t>
+  </si>
+  <si>
+    <t>IsPressedKeyShift()</t>
+  </si>
+  <si>
+    <t>IsShift()</t>
+  </si>
+  <si>
+    <t>IsPressedKeyCtrl()</t>
+  </si>
+  <si>
+    <t>IsCtrl()</t>
+  </si>
+  <si>
+    <t>SetButtKeyFlags()</t>
+  </si>
+  <si>
+    <t>SetButtonKeyFlags()</t>
+  </si>
+  <si>
+    <t>Tên sai (private)</t>
+  </si>
+  <si>
+    <t>Methods — cần thêm mới (từ CMouse)</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Loại</t>
+  </si>
+  <si>
+    <t>Mục đích</t>
+  </si>
+  <si>
+    <t>CheckChangeLeftButtonState(string)</t>
+  </si>
+  <si>
+    <t>private</t>
+  </si>
+  <si>
+    <r>
+      <t>Detect change + fire </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="163"/>
+      </rPr>
+      <t>ON_CHANGE_MOUSE_LEFT_BUTTON</t>
+    </r>
+  </si>
+  <si>
+    <t>CheckDoubleClick()</t>
+  </si>
+  <si>
+    <r>
+      <t>Detect double-click + fire </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="163"/>
+      </rPr>
+      <t>ON_DOUBLE_CLICK</t>
+    </r>
+  </si>
+  <si>
+    <t>public getter</t>
+  </si>
+  <si>
+    <r>
+      <t>Trả về </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <color rgb="FFA31515"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+        <charset val="163"/>
+      </rPr>
+      <t>m_left_button_state</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -898,6 +1109,14 @@
       <color rgb="FFA31515"/>
       <name val="Courier New"/>
       <family val="3"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color rgb="FF616161"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
       <charset val="163"/>
     </font>
   </fonts>
@@ -953,7 +1172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -975,6 +1194,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2633,4 +2855,360 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09A35452-178D-48B8-91E5-F29D7EAEDFD6}">
+  <dimension ref="A2:D33"/>
+  <sheetFormatPr defaultColWidth="19.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="42.21875" customWidth="1"/>
+    <col min="2" max="2" width="46.5546875" customWidth="1"/>
+    <col min="3" max="3" width="59.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+    </row>
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+    </row>
+    <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A28" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+    </row>
+    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A28:D28"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>